<commit_message>
Strengthen Coin Survivor QA cases and balance input validation
</commit_message>
<xml_diff>
--- a/balance/project2-balance-v5-ko.xlsx
+++ b/balance/project2-balance-v5-ko.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="대시보드" sheetId="1" r:id="Rb626d8972d274b93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="현재 기준" sheetId="2" r:id="Rb74703873c784c44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="성장 곡선" sheetId="3" r:id="R50504a24ab594f3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="스폰 타임라인" sheetId="4" r:id="R76bfe98f8c9948af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="적·보스" sheetId="5" r:id="R8485f3498e994310"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="경제 흐름" sheetId="6" r:id="R7399d7a6887d4318"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="인벤토리 경제" sheetId="7" r:id="R02a326f0ff9c4ef8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="패시브 시너지" sheetId="8" r:id="R29390b7de19e4538"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="무기 DPS" sheetId="9" r:id="R27b62de1b25048ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="성장·카메라 예산" sheetId="10" r:id="Rbb5ae4810cb34868"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="플레이 모드 입력" sheetId="11" r:id="Rfed1188727df484d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="데이터 품질" sheetId="12" r:id="Rcc886a2e5852456a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="대시보드" sheetId="1" r:id="R1578d9b0fb3041ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="현재 기준" sheetId="2" r:id="R835590ebbe6344ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="성장 곡선" sheetId="3" r:id="R37b5017548bd44b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="스폰 타임라인" sheetId="4" r:id="Rba8d216dbc084452"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="적·보스" sheetId="5" r:id="Rf370b4e3a16f4b08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="경제 흐름" sheetId="6" r:id="R03491c0fa278440b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="인벤토리 경제" sheetId="7" r:id="R219ee3e3d94e4b7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="패시브 시너지" sheetId="8" r:id="R44560722afae4e4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="무기 DPS" sheetId="9" r:id="R0f4ff1ad4d1141c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="성장·카메라 예산" sheetId="10" r:id="Rf3a6a09207094051"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="플레이 모드 입력" sheetId="11" r:id="R8724e8e7b0684cb0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="데이터 품질" sheetId="12" r:id="R0cc94dde553f47f0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -201,7 +201,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -211,7 +211,7 @@
         <x:b/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -221,7 +221,7 @@
         <x:b/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -231,7 +231,7 @@
         <x:b/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -242,7 +242,7 @@
 
 <file path=xl/drawings/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <c:lang val="ko-KR"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <c:chart>
     <c:title>
@@ -252,7 +252,7 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:rPr lang="ko-KR" sz="1200">
+              <a:rPr sz="1200">
                 <a:latin typeface="맑은 고딕"/>
                 <a:ea typeface="맑은 고딕"/>
                 <a:cs typeface="맑은 고딕"/>
@@ -263,27 +263,23 @@
         </c:rich>
       </c:tx>
       <c:txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
         <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr lang="ko-KR" sz="1200">
+            <a:defRPr sz="1200">
               <a:latin typeface="맑은 고딕"/>
               <a:ea typeface="맑은 고딕"/>
               <a:cs typeface="맑은 고딕"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="ko-KR" sz="1200">
-            <a:latin typeface="맑은 고딕"/>
-            <a:ea typeface="맑은 고딕"/>
-            <a:cs typeface="맑은 고딕"/>
-          </a:endParaRPr>
         </a:p>
       </c:txPr>
     </c:title>
     <c:plotArea>
       <c:lineChart>
         <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
@@ -363,27 +359,20 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr lang="ko-KR" sz="900">
+              <a:defRPr sz="900">
                 <a:latin typeface="맑은 고딕"/>
                 <a:ea typeface="맑은 고딕"/>
                 <a:cs typeface="맑은 고딕"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="ko-KR" sz="900">
-              <a:latin typeface="맑은 고딕"/>
-              <a:ea typeface="맑은 고딕"/>
-              <a:cs typeface="맑은 고딕"/>
-            </a:endParaRPr>
           </a:p>
         </c:txPr>
         <c:crossAx val="48672768"/>
-        <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
         <c:axId val="48672768"/>
@@ -406,21 +395,16 @@
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr lang="ko-KR" sz="900">
+              <a:defRPr sz="900">
                 <a:latin typeface="맑은 고딕"/>
                 <a:ea typeface="맑은 고딕"/>
                 <a:cs typeface="맑은 고딕"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="ko-KR" sz="900">
-              <a:latin typeface="맑은 고딕"/>
-              <a:ea typeface="맑은 고딕"/>
-              <a:cs typeface="맑은 고딕"/>
-            </a:endParaRPr>
           </a:p>
         </c:txPr>
         <c:crossAx val="48650112"/>
@@ -431,21 +415,16 @@
       <c:legendPos val="b"/>
       <c:overlay val="0"/>
       <c:txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
         <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr lang="ko-KR" sz="1000">
+            <a:defRPr sz="1000">
               <a:latin typeface="맑은 고딕"/>
               <a:ea typeface="맑은 고딕"/>
               <a:cs typeface="맑은 고딕"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="ko-KR" sz="1000">
-            <a:latin typeface="맑은 고딕"/>
-            <a:ea typeface="맑은 고딕"/>
-            <a:cs typeface="맑은 고딕"/>
-          </a:endParaRPr>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -464,7 +443,7 @@
 
 <file path=xl/drawings/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <c:lang val="ko-KR"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <c:chart>
     <c:title>
@@ -474,7 +453,7 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:rPr lang="ko-KR" sz="1200">
+              <a:rPr sz="1200">
                 <a:latin typeface="맑은 고딕"/>
                 <a:ea typeface="맑은 고딕"/>
                 <a:cs typeface="맑은 고딕"/>
@@ -485,27 +464,23 @@
         </c:rich>
       </c:tx>
       <c:txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
         <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr lang="ko-KR" sz="1200">
+            <a:defRPr sz="1200">
               <a:latin typeface="맑은 고딕"/>
               <a:ea typeface="맑은 고딕"/>
               <a:cs typeface="맑은 고딕"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="ko-KR" sz="1200">
-            <a:latin typeface="맑은 고딕"/>
-            <a:ea typeface="맑은 고딕"/>
-            <a:cs typeface="맑은 고딕"/>
-          </a:endParaRPr>
         </a:p>
       </c:txPr>
     </c:title>
     <c:plotArea>
       <c:lineChart>
         <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
@@ -612,27 +587,20 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr lang="ko-KR" sz="900">
+              <a:defRPr sz="900">
                 <a:latin typeface="맑은 고딕"/>
                 <a:ea typeface="맑은 고딕"/>
                 <a:cs typeface="맑은 고딕"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="ko-KR" sz="900">
-              <a:latin typeface="맑은 고딕"/>
-              <a:ea typeface="맑은 고딕"/>
-              <a:cs typeface="맑은 고딕"/>
-            </a:endParaRPr>
           </a:p>
         </c:txPr>
         <c:crossAx val="48672768"/>
-        <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
         <c:axId val="48672768"/>
@@ -655,21 +623,16 @@
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr lang="ko-KR" sz="900">
+              <a:defRPr sz="900">
                 <a:latin typeface="맑은 고딕"/>
                 <a:ea typeface="맑은 고딕"/>
                 <a:cs typeface="맑은 고딕"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="ko-KR" sz="900">
-              <a:latin typeface="맑은 고딕"/>
-              <a:ea typeface="맑은 고딕"/>
-              <a:cs typeface="맑은 고딕"/>
-            </a:endParaRPr>
           </a:p>
         </c:txPr>
         <c:crossAx val="48650112"/>
@@ -680,21 +643,16 @@
       <c:legendPos val="b"/>
       <c:overlay val="0"/>
       <c:txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
         <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr lang="ko-KR" sz="1000">
+            <a:defRPr sz="1000">
               <a:latin typeface="맑은 고딕"/>
               <a:ea typeface="맑은 고딕"/>
               <a:cs typeface="맑은 고딕"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="ko-KR" sz="1000">
-            <a:latin typeface="맑은 고딕"/>
-            <a:ea typeface="맑은 고딕"/>
-            <a:cs typeface="맑은 고딕"/>
-          </a:endParaRPr>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -713,7 +671,7 @@
 
 <file path=xl/drawings/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <c:lang val="ko-KR"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <c:chart>
     <c:title>
@@ -723,7 +681,7 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:rPr lang="ko-KR" sz="1200">
+              <a:rPr sz="1200">
                 <a:latin typeface="맑은 고딕"/>
                 <a:ea typeface="맑은 고딕"/>
                 <a:cs typeface="맑은 고딕"/>
@@ -734,21 +692,16 @@
         </c:rich>
       </c:tx>
       <c:txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
         <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr lang="ko-KR" sz="1200">
+            <a:defRPr sz="1200">
               <a:latin typeface="맑은 고딕"/>
               <a:ea typeface="맑은 고딕"/>
               <a:cs typeface="맑은 고딕"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="ko-KR" sz="1200">
-            <a:latin typeface="맑은 고딕"/>
-            <a:ea typeface="맑은 고딕"/>
-            <a:cs typeface="맑은 고딕"/>
-          </a:endParaRPr>
         </a:p>
       </c:txPr>
     </c:title>
@@ -805,27 +758,20 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr lang="ko-KR" sz="900">
+              <a:defRPr sz="900">
                 <a:latin typeface="맑은 고딕"/>
                 <a:ea typeface="맑은 고딕"/>
                 <a:cs typeface="맑은 고딕"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="ko-KR" sz="900">
-              <a:latin typeface="맑은 고딕"/>
-              <a:ea typeface="맑은 고딕"/>
-              <a:cs typeface="맑은 고딕"/>
-            </a:endParaRPr>
           </a:p>
         </c:txPr>
         <c:crossAx val="48672768"/>
-        <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
         <c:axId val="48672768"/>
@@ -848,21 +794,16 @@
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr lang="ko-KR" sz="900">
+              <a:defRPr sz="900">
                 <a:latin typeface="맑은 고딕"/>
                 <a:ea typeface="맑은 고딕"/>
                 <a:cs typeface="맑은 고딕"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="ko-KR" sz="900">
-              <a:latin typeface="맑은 고딕"/>
-              <a:ea typeface="맑은 고딕"/>
-              <a:cs typeface="맑은 고딕"/>
-            </a:endParaRPr>
           </a:p>
         </c:txPr>
         <c:crossAx val="48650112"/>
@@ -908,7 +849,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R39695f006c5a4022"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R343edeb216cd4ca5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -943,7 +884,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re56b434e4b1d4098"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R87ff405c88d74780"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -978,7 +919,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra9712e048c454d28"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R57fe031058504c48"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1194,7 +1135,7 @@
   <x:sheetData>
     <x:row r="1" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>Coin Survivor 밸런스 계약 v5</x:v>
+        <x:v>Coin Survivor 밸런스 조정안 v5</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>
@@ -1204,9 +1145,9 @@
       <x:c r="G1" s="3"/>
       <x:c r="H1" s="3"/>
     </x:row>
-    <x:row r="2" ht="15" hidden="0" customHeight="1">
+    <x:row r="2" ht="50" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>코드 기준과 Play Mode 실측을 분리합니다. 빈 실측값은 통과가 아니라 미측정입니다.</x:v>
+        <x:v>114G에서 상품 네 개(40G)를 사면 74G가 남아 100G 확장을 선택할 수 없었습니다. 구매와 확장을 함께 선택할 여유를 주는 방향을 검토했습니다.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -1219,7 +1160,7 @@
     <x:row r="3"/>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="8" t="str">
-        <x:v>이번 패치의 철학</x:v>
+        <x:v>비용과 성장 흐름의 조정 목표</x:v>
       </x:c>
       <x:c r="B4" s="8"/>
       <x:c r="C4" s="8"/>
@@ -1310,13 +1251,13 @@
         <x:v>스폰 증가로 프레임 급락</x:v>
       </x:c>
       <x:c r="D10" s="12" t="str">
-        <x:v>15분 단일 통합 런</x:v>
+        <x:v>15분 플레이 측정</x:v>
       </x:c>
     </x:row>
     <x:row r="11"/>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="8" t="str">
-        <x:v>코드 적용 상태와 다음 검증 경계</x:v>
+        <x:v>2026년 7월 16일 기준 수치와 확인 항목</x:v>
       </x:c>
       <x:c r="B12" s="8"/>
       <x:c r="C12" s="8"/>
@@ -1416,7 +1357,7 @@
         <x:v>통합 Play Mode</x:v>
       </x:c>
       <x:c r="B18" s="12" t="str">
-        <x:v>사용자 수행 전</x:v>
+        <x:v>입력 전</x:v>
       </x:c>
       <x:c r="C18" s="12" t="str">
         <x:v>신규 콘솔 오류 0</x:v>
@@ -1425,7 +1366,7 @@
         <x:v>미측정</x:v>
       </x:c>
       <x:c r="E18" s="12" t="str">
-        <x:v>체크리스트를 다음 단계에서 실행</x:v>
+        <x:v>15분 플레이 결과 입력</x:v>
       </x:c>
     </x:row>
     <x:row r="19"/>
@@ -1603,7 +1544,7 @@
   <x:sheetData>
     <x:row r="1" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>몸집 성장·카메라·판정 상태 계약</x:v>
+        <x:v>몸집 성장·카메라·판정 상태</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>
@@ -1970,7 +1911,7 @@
   <x:sheetData>
     <x:row r="1" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>단일 통합 Play Mode 입력</x:v>
+        <x:v>플레이 측정 기록</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>
@@ -1986,9 +1927,9 @@
       <x:c r="M1" s="3"/>
       <x:c r="N1" s="3"/>
     </x:row>
-    <x:row r="2" ht="15" hidden="0" customHeight="1">
+    <x:row r="2" ht="36" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>사용자 검증 단계에서 노란 셀만 입력합니다. 지금은 전부 미측정이 정상입니다.</x:v>
+        <x:v>노란 칸에 실제 측정값을 입력합니다. 판정에 필요한 원거리 적 수, 화면 안·밖 피해, FPS, 1% low, 오류 수가 모두 숫자여야 판정합니다.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -2066,7 +2007,7 @@
       <x:c r="L5" s="16"/>
       <x:c r="M5" s="16"/>
       <x:c r="N5" s="12" t="str">
-        <x:f>IF(COUNT(B5:M5)=0,"미측정",IF(AND(G5&lt;=6,K5&gt;=55,L5&gt;=45,M5=0,IF(I5+J5=0,FALSE,I5/(I5+J5)&gt;=0.8)),"목표 범위","재조정"))</x:f>
+        <x:f>IF(COUNT(G5,I5,J5,K5,L5,M5)&lt;6,"미측정",IF(AND(G5&lt;=6,K5&gt;=55,L5&gt;=45,M5=0,IF(I5+J5=0,FALSE,I5/(I5+J5)&gt;=0.8)),"목표 범위","재조정"))</x:f>
         <x:v>미측정</x:v>
       </x:c>
     </x:row>
@@ -2087,7 +2028,7 @@
       <x:c r="L6" s="16"/>
       <x:c r="M6" s="16"/>
       <x:c r="N6" s="12" t="str">
-        <x:f>IF(COUNT(B6:M6)=0,"미측정",IF(AND(G6&lt;=6,K6&gt;=55,L6&gt;=45,M6=0,IF(I6+J6=0,FALSE,I6/(I6+J6)&gt;=0.8)),"목표 범위","재조정"))</x:f>
+        <x:f>IF(COUNT(G6,I6,J6,K6,L6,M6)&lt;6,"미측정",IF(AND(G6&lt;=6,K6&gt;=55,L6&gt;=45,M6=0,IF(I6+J6=0,FALSE,I6/(I6+J6)&gt;=0.8)),"목표 범위","재조정"))</x:f>
         <x:v>미측정</x:v>
       </x:c>
     </x:row>
@@ -2108,7 +2049,7 @@
       <x:c r="L7" s="16"/>
       <x:c r="M7" s="16"/>
       <x:c r="N7" s="12" t="str">
-        <x:f>IF(COUNT(B7:M7)=0,"미측정",IF(AND(G7&lt;=6,K7&gt;=55,L7&gt;=45,M7=0,IF(I7+J7=0,FALSE,I7/(I7+J7)&gt;=0.8)),"목표 범위","재조정"))</x:f>
+        <x:f>IF(COUNT(G7,I7,J7,K7,L7,M7)&lt;6,"미측정",IF(AND(G7&lt;=6,K7&gt;=55,L7&gt;=45,M7=0,IF(I7+J7=0,FALSE,I7/(I7+J7)&gt;=0.8)),"목표 범위","재조정"))</x:f>
         <x:v>미측정</x:v>
       </x:c>
     </x:row>
@@ -2129,7 +2070,7 @@
       <x:c r="L8" s="16"/>
       <x:c r="M8" s="16"/>
       <x:c r="N8" s="12" t="str">
-        <x:f>IF(COUNT(B8:M8)=0,"미측정",IF(AND(G8&lt;=6,K8&gt;=55,L8&gt;=45,M8=0,IF(I8+J8=0,FALSE,I8/(I8+J8)&gt;=0.8)),"목표 범위","재조정"))</x:f>
+        <x:f>IF(COUNT(G8,I8,J8,K8,L8,M8)&lt;6,"미측정",IF(AND(G8&lt;=6,K8&gt;=55,L8&gt;=45,M8=0,IF(I8+J8=0,FALSE,I8/(I8+J8)&gt;=0.8)),"목표 범위","재조정"))</x:f>
         <x:v>미측정</x:v>
       </x:c>
     </x:row>
@@ -2150,7 +2091,7 @@
       <x:c r="L9" s="16"/>
       <x:c r="M9" s="16"/>
       <x:c r="N9" s="12" t="str">
-        <x:f>IF(COUNT(B9:M9)=0,"미측정",IF(AND(G9&lt;=6,K9&gt;=55,L9&gt;=45,M9=0,IF(I9+J9=0,FALSE,I9/(I9+J9)&gt;=0.8)),"목표 범위","재조정"))</x:f>
+        <x:f>IF(COUNT(G9,I9,J9,K9,L9,M9)&lt;6,"미측정",IF(AND(G9&lt;=6,K9&gt;=55,L9&gt;=45,M9=0,IF(I9+J9=0,FALSE,I9/(I9+J9)&gt;=0.8)),"목표 범위","재조정"))</x:f>
         <x:v>미측정</x:v>
       </x:c>
     </x:row>
@@ -2171,7 +2112,7 @@
       <x:c r="L10" s="16"/>
       <x:c r="M10" s="16"/>
       <x:c r="N10" s="12" t="str">
-        <x:f>IF(COUNT(B10:M10)=0,"미측정",IF(AND(G10&lt;=6,K10&gt;=55,L10&gt;=45,M10=0,IF(I10+J10=0,FALSE,I10/(I10+J10)&gt;=0.8)),"목표 범위","재조정"))</x:f>
+        <x:f>IF(COUNT(G10,I10,J10,K10,L10,M10)&lt;6,"미측정",IF(AND(G10&lt;=6,K10&gt;=55,L10&gt;=45,M10=0,IF(I10+J10=0,FALSE,I10/(I10+J10)&gt;=0.8)),"목표 범위","재조정"))</x:f>
         <x:v>미측정</x:v>
       </x:c>
     </x:row>
@@ -2192,7 +2133,7 @@
       <x:c r="L11" s="16"/>
       <x:c r="M11" s="16"/>
       <x:c r="N11" s="12" t="str">
-        <x:f>IF(COUNT(B11:M11)=0,"미측정",IF(AND(G11&lt;=6,K11&gt;=55,L11&gt;=45,M11=0,IF(I11+J11=0,FALSE,I11/(I11+J11)&gt;=0.8)),"목표 범위","재조정"))</x:f>
+        <x:f>IF(COUNT(G11,I11,J11,K11,L11,M11)&lt;6,"미측정",IF(AND(G11&lt;=6,K11&gt;=55,L11&gt;=45,M11=0,IF(I11+J11=0,FALSE,I11/(I11+J11)&gt;=0.8)),"목표 범위","재조정"))</x:f>
         <x:v>미측정</x:v>
       </x:c>
     </x:row>
@@ -2213,7 +2154,7 @@
       <x:c r="L12" s="16"/>
       <x:c r="M12" s="16"/>
       <x:c r="N12" s="12" t="str">
-        <x:f>IF(COUNT(B12:M12)=0,"미측정",IF(AND(G12&lt;=6,K12&gt;=55,L12&gt;=45,M12=0,IF(I12+J12=0,FALSE,I12/(I12+J12)&gt;=0.8)),"목표 범위","재조정"))</x:f>
+        <x:f>IF(COUNT(G12,I12,J12,K12,L12,M12)&lt;6,"미측정",IF(AND(G12&lt;=6,K12&gt;=55,L12&gt;=45,M12=0,IF(I12+J12=0,FALSE,I12/(I12+J12)&gt;=0.8)),"목표 범위","재조정"))</x:f>
         <x:v>미측정</x:v>
       </x:c>
     </x:row>
@@ -2234,7 +2175,7 @@
       <x:c r="L13" s="16"/>
       <x:c r="M13" s="16"/>
       <x:c r="N13" s="12" t="str">
-        <x:f>IF(COUNT(B13:M13)=0,"미측정",IF(AND(G13&lt;=6,K13&gt;=55,L13&gt;=45,M13=0,IF(I13+J13=0,FALSE,I13/(I13+J13)&gt;=0.8)),"목표 범위","재조정"))</x:f>
+        <x:f>IF(COUNT(G13,I13,J13,K13,L13,M13)&lt;6,"미측정",IF(AND(G13&lt;=6,K13&gt;=55,L13&gt;=45,M13=0,IF(I13+J13=0,FALSE,I13/(I13+J13)&gt;=0.8)),"목표 범위","재조정"))</x:f>
         <x:v>미측정</x:v>
       </x:c>
     </x:row>
@@ -2467,7 +2408,7 @@
         <x:v>남은 위험</x:v>
       </x:c>
       <x:c r="G4" s="15" t="str">
-        <x:v>담당</x:v>
+        <x:v>확인 방식</x:v>
       </x:c>
       <x:c r="H4" s="15" t="str">
         <x:v>갱신 규칙</x:v>
@@ -2493,7 +2434,7 @@
         <x:v>Play Mode 체감</x:v>
       </x:c>
       <x:c r="G5" s="12" t="str">
-        <x:v>Codex</x:v>
+        <x:v>코드·데이터 분석</x:v>
       </x:c>
       <x:c r="H5" s="12" t="str">
         <x:v>코드 변경 시</x:v>
@@ -2519,7 +2460,7 @@
         <x:v>실제 alive 변동</x:v>
       </x:c>
       <x:c r="G6" s="12" t="str">
-        <x:v>Codex</x:v>
+        <x:v>코드·데이터 분석</x:v>
       </x:c>
       <x:c r="H6" s="12" t="str">
         <x:v>스폰 변경 시</x:v>
@@ -2545,7 +2486,7 @@
         <x:v>런타임 참조</x:v>
       </x:c>
       <x:c r="G7" s="12" t="str">
-        <x:v>Codex</x:v>
+        <x:v>코드·데이터 분석</x:v>
       </x:c>
       <x:c r="H7" s="12" t="str">
         <x:v>가격 변경 시</x:v>
@@ -2559,19 +2500,19 @@
         <x:v>NotoSansKR TMP assets</x:v>
       </x:c>
       <x:c r="C8" s="12" t="str">
-        <x:v>사용자 제외</x:v>
+        <x:v>표시 확인</x:v>
       </x:c>
       <x:c r="D8" s="12" t="str">
-        <x:v>체크인 제외</x:v>
+        <x:v>별도 확인 기록</x:v>
       </x:c>
       <x:c r="E8" s="12" t="str">
-        <x:v>Start 화면 사용자 확인</x:v>
+        <x:v>업그레이드 화면 한글 확인</x:v>
       </x:c>
       <x:c r="F8" s="12" t="str">
-        <x:v>다른 씬 fallback</x:v>
+        <x:v>다른 화면의 표시</x:v>
       </x:c>
       <x:c r="G8" s="12" t="str">
-        <x:v>사용자</x:v>
+        <x:v>직접 플레이</x:v>
       </x:c>
       <x:c r="H8" s="12" t="str">
         <x:v>별도 폰트 작업</x:v>
@@ -2591,13 +2532,13 @@
         <x:v>미측정</x:v>
       </x:c>
       <x:c r="E9" s="12" t="str">
-        <x:v>15분 통합 런</x:v>
+        <x:v>15분 플레이 측정</x:v>
       </x:c>
       <x:c r="F9" s="12" t="str">
         <x:v>무기별 샘플 부족</x:v>
       </x:c>
       <x:c r="G9" s="12" t="str">
-        <x:v>사용자</x:v>
+        <x:v>플레이 측정</x:v>
       </x:c>
       <x:c r="H9" s="12" t="str">
         <x:v>매 밸패</x:v>
@@ -2617,13 +2558,13 @@
         <x:v>미측정</x:v>
       </x:c>
       <x:c r="E10" s="12" t="str">
-        <x:v>동일 PC 15분 런</x:v>
+        <x:v>동일 PC 15분 측정</x:v>
       </x:c>
       <x:c r="F10" s="12" t="str">
         <x:v>환경 의존</x:v>
       </x:c>
       <x:c r="G10" s="12" t="str">
-        <x:v>사용자</x:v>
+        <x:v>플레이 측정</x:v>
       </x:c>
       <x:c r="H10" s="12" t="str">
         <x:v>스폰/투사체 변경 시</x:v>
@@ -2649,7 +2590,7 @@
         <x:v>정적 재현 불가</x:v>
       </x:c>
       <x:c r="G11" s="12" t="str">
-        <x:v>사용자</x:v>
+        <x:v>플레이 확인</x:v>
       </x:c>
       <x:c r="H11" s="12" t="str">
         <x:v>맵/풀링 변경 시</x:v>
@@ -2659,7 +2600,7 @@
     <x:row r="13"/>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="8" t="str">
-        <x:v>통과 기준</x:v>
+        <x:v>확인 범위</x:v>
       </x:c>
       <x:c r="B14" s="8"/>
       <x:c r="C14" s="8"/>
@@ -2674,13 +2615,13 @@
         <x:v>검증 층</x:v>
       </x:c>
       <x:c r="B15" s="15" t="str">
-        <x:v>이번 목표에서 완료</x:v>
+        <x:v>확인한 내용</x:v>
       </x:c>
       <x:c r="C15" s="15" t="str">
-        <x:v>이번 목표에서 완료 아님</x:v>
+        <x:v>추가 확인 대상</x:v>
       </x:c>
       <x:c r="D15" s="15" t="str">
-        <x:v>완료 표기 규칙</x:v>
+        <x:v>기록 방법</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
@@ -2688,7 +2629,7 @@
         <x:v>정적/컴파일</x:v>
       </x:c>
       <x:c r="B16" s="12" t="str">
-        <x:v>C# 0 오류·0 경고, 참조/충돌 스캔</x:v>
+        <x:v>코드·참조·컴파일 점검</x:v>
       </x:c>
       <x:c r="C16" s="12" t="str">
         <x:v>게임 체감</x:v>
@@ -2702,10 +2643,10 @@
         <x:v>Play Mode</x:v>
       </x:c>
       <x:c r="B17" s="12" t="str">
-        <x:v>체크리스트 설계까지</x:v>
+        <x:v>측정 항목과 입력 양식</x:v>
       </x:c>
       <x:c r="C17" s="12" t="str">
-        <x:v>사용자의 실제 15분 런</x:v>
+        <x:v>실제 플레이 측정값</x:v>
       </x:c>
       <x:c r="D17" s="12" t="str">
         <x:v>입력 전에는 항상 미측정</x:v>
@@ -2713,16 +2654,16 @@
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="12" t="str">
-        <x:v>제출</x:v>
+        <x:v>기준 버전</x:v>
       </x:c>
       <x:c r="B18" s="12" t="str">
-        <x:v>폰트 제외 Plastic 체크인</x:v>
+        <x:v>2026년 7월 16일 작업 기록</x:v>
       </x:c>
       <x:c r="C18" s="12" t="str">
-        <x:v>Play Mode 승인</x:v>
+        <x:v>현재 버전의 실행 결과</x:v>
       </x:c>
       <x:c r="D18" s="12" t="str">
-        <x:v>체크인 changeset 기록</x:v>
+        <x:v>기준 날짜와 별도로 기록</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3677,7 +3618,7 @@
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="위험"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R950c2861f35c44a8"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8e3f27969e34d4e"/>
 </x:worksheet>
 </file>
 
@@ -4786,7 +4727,7 @@
     <x:cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="원거리"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e5b24a9596c4358"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c5dd1e3bfa54ecc"/>
 </x:worksheet>
 </file>
 
@@ -5383,7 +5324,7 @@
     <x:mergeCell ref="A2:L2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9598c9b1fb974b18"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8010b5ff45d04006"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Shorten balance sheet labels for readability
</commit_message>
<xml_diff>
--- a/balance/project2-balance-v5-ko.xlsx
+++ b/balance/project2-balance-v5-ko.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="대시보드" sheetId="1" r:id="R1578d9b0fb3041ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="현재 기준" sheetId="2" r:id="R835590ebbe6344ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="성장 곡선" sheetId="3" r:id="R37b5017548bd44b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="스폰 타임라인" sheetId="4" r:id="Rba8d216dbc084452"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="적·보스" sheetId="5" r:id="Rf370b4e3a16f4b08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="경제 흐름" sheetId="6" r:id="R03491c0fa278440b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="인벤토리 경제" sheetId="7" r:id="R219ee3e3d94e4b7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="패시브 시너지" sheetId="8" r:id="R44560722afae4e4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="무기 DPS" sheetId="9" r:id="R0f4ff1ad4d1141c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="성장·카메라 예산" sheetId="10" r:id="Rf3a6a09207094051"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="플레이 모드 입력" sheetId="11" r:id="R8724e8e7b0684cb0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="데이터 품질" sheetId="12" r:id="R0cc94dde553f47f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="대시보드" sheetId="1" r:id="R2bd09e3ad9604f3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="현재 기준" sheetId="2" r:id="R1818d475c89842c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="성장 곡선" sheetId="3" r:id="Reaff7a6628a3481c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="스폰 타임라인" sheetId="4" r:id="R0b40bdbe2b7d41cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="적·보스" sheetId="5" r:id="R6309a79fad9a497a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="경제 흐름" sheetId="6" r:id="R092807b079704e18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="인벤토리 경제" sheetId="7" r:id="R3f0627cd3a004d9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="패시브 시너지" sheetId="8" r:id="R3ab8fb6c97944d26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="무기 DPS" sheetId="9" r:id="R2da7ebb02cf94b40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="성장·카메라 예산" sheetId="10" r:id="R5c6945b8375a43f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="플레이 모드 입력" sheetId="11" r:id="Ra6c6f0ad9bde4662"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="데이터 품질" sheetId="12" r:id="R899b67e3a247405c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -849,7 +849,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R343edeb216cd4ca5"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R846b538c58ea4fa1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -884,7 +884,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R87ff405c88d74780"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb5e9b5da76904e67"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -919,7 +919,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R57fe031058504c48"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re1182f34dc06430d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2434,7 +2434,7 @@
         <x:v>Play Mode 체감</x:v>
       </x:c>
       <x:c r="G5" s="12" t="str">
-        <x:v>코드·데이터 분석</x:v>
+        <x:v>코드 분석</x:v>
       </x:c>
       <x:c r="H5" s="12" t="str">
         <x:v>코드 변경 시</x:v>
@@ -2460,7 +2460,7 @@
         <x:v>실제 alive 변동</x:v>
       </x:c>
       <x:c r="G6" s="12" t="str">
-        <x:v>코드·데이터 분석</x:v>
+        <x:v>코드 분석</x:v>
       </x:c>
       <x:c r="H6" s="12" t="str">
         <x:v>스폰 변경 시</x:v>
@@ -2486,7 +2486,7 @@
         <x:v>런타임 참조</x:v>
       </x:c>
       <x:c r="G7" s="12" t="str">
-        <x:v>코드·데이터 분석</x:v>
+        <x:v>코드 분석</x:v>
       </x:c>
       <x:c r="H7" s="12" t="str">
         <x:v>가격 변경 시</x:v>
@@ -3618,7 +3618,7 @@
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="위험"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8e3f27969e34d4e"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Recca1801bbc048a6"/>
 </x:worksheet>
 </file>
 
@@ -4727,7 +4727,7 @@
     <x:cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="원거리"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c5dd1e3bfa54ecc"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62f56c769aaa4288"/>
 </x:worksheet>
 </file>
 
@@ -5324,7 +5324,7 @@
     <x:mergeCell ref="A2:L2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8010b5ff45d04006"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf18fb57988d84f39"/>
 </x:worksheet>
 </file>
 

</xml_diff>